<commit_message>
WifiWeather display and ST77xx that runs on UNOr4
</commit_message>
<xml_diff>
--- a/arduino_uno_r4.xlsx
+++ b/arduino_uno_r4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\UNOR4-stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4997D2B-A068-4648-B657-4735A902C82E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{029698A8-AF9D-4CCE-8BFD-BEDCDD6E6988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="840" yWindow="2745" windowWidth="19845" windowHeight="14340" activeTab="3" xr2:uid="{8DF1AF20-4F17-4E13-BB05-CAA1D9B0E58D}"/>
+    <workbookView xWindow="1995" yWindow="540" windowWidth="29535" windowHeight="18630" activeTab="1" xr2:uid="{8DF1AF20-4F17-4E13-BB05-CAA1D9B0E58D}"/>
   </bookViews>
   <sheets>
     <sheet name="Table033 (Page 23-26)" sheetId="2" r:id="rId1"/>
@@ -24,7 +24,6 @@
     <definedName name="ExternalData_1" localSheetId="1" hidden="1">Wifi!$D$1:$U$40</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>